<commit_message>
fix skills in data_FOR_CHECK.xlsx
</commit_message>
<xml_diff>
--- a/public/data_FOR_CHECK.xlsx
+++ b/public/data_FOR_CHECK.xlsx
@@ -14173,7 +14173,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z342"/>
+  <dimension ref="A1:AA342"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -14252,6 +14252,9 @@
         <v>Aspiration</v>
       </c>
       <c r="Z1" t="str">
+        <v>Skills</v>
+      </c>
+      <c r="AA1" t="str">
         <v>relativesIds</v>
       </c>
     </row>
@@ -14331,6 +14334,9 @@
       <c r="Y2" t="str">
         <v>Renaissance Sim</v>
       </c>
+      <c r="Z2" t="str">
+        <v>Writing4</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -14405,6 +14411,9 @@
       <c r="Y3" t="str">
         <v>Party Animal</v>
       </c>
+      <c r="Z3" t="str">
+        <v>Charisma2,Fitness2,Programming2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -14470,6 +14479,9 @@
       <c r="Y4" t="str">
         <v>Musical Genius</v>
       </c>
+      <c r="Z4" t="str">
+        <v>Violin2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -14535,6 +14547,9 @@
       <c r="Y5" t="str">
         <v>Whiz Kid</v>
       </c>
+      <c r="Z5" t="str">
+        <v>Creativity1,Mental1,Motor1,Social1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -14606,7 +14621,7 @@
       <c r="Y6" t="str">
         <v>Successful Lineage</v>
       </c>
-      <c r="Z6" t="str">
+      <c r="AA6" t="str">
         <v>LewisVivian,LewisEric</v>
       </c>
     </row>
@@ -14680,7 +14695,7 @@
       <c r="Y7" t="str">
         <v>Big Happy Family</v>
       </c>
-      <c r="Z7" t="str">
+      <c r="AA7" t="str">
         <v>KimDennis,KimSpencerAlice</v>
       </c>
     </row>
@@ -14742,7 +14757,7 @@
       <c r="T8" t="str">
         <v/>
       </c>
-      <c r="Z8" t="str">
+      <c r="AA8" t="str">
         <v>LewisVivian</v>
       </c>
     </row>
@@ -14819,7 +14834,7 @@
       <c r="Y9" t="str">
         <v>Mansion Baron</v>
       </c>
-      <c r="Z9" t="str">
+      <c r="AA9" t="str">
         <v>KimDennis</v>
       </c>
     </row>
@@ -17593,7 +17608,7 @@
       <c r="R70" t="str">
         <v>VatoreCaleb</v>
       </c>
-      <c r="Z70" t="str">
+      <c r="AA70" t="str">
         <v>ZhuLily</v>
       </c>
     </row>
@@ -17637,7 +17652,7 @@
       <c r="R71" t="str">
         <v>VatoreLilith</v>
       </c>
-      <c r="Z71" t="str">
+      <c r="AA71" t="str">
         <v>ZhuLily</v>
       </c>
     </row>
@@ -18335,7 +18350,7 @@
       <c r="M87" t="str">
         <v>AltoHolly</v>
       </c>
-      <c r="Z87" t="str">
+      <c r="AA87" t="str">
         <v>AltoEnzo</v>
       </c>
     </row>
@@ -20218,7 +20233,7 @@
       <c r="M208" t="str">
         <v>ZhuLily</v>
       </c>
-      <c r="Z208" t="str">
+      <c r="AA208" t="str">
         <v>VatoreLilith,VatoreCaleb</v>
       </c>
     </row>
@@ -21825,7 +21840,7 @@
       <c r="S320" t="str">
         <v>CappConsort</v>
       </c>
-      <c r="Z320" t="str">
+      <c r="AA320" t="str">
         <v>CappBeatrice,CappBeatrice,CappVirgilio</v>
       </c>
     </row>
@@ -21913,7 +21928,7 @@
       <c r="Q322" t="str">
         <v>MontyRomeo,MontyJuliette</v>
       </c>
-      <c r="Z322" t="str">
+      <c r="AA322" t="str">
         <v>CappTybalt,CappBeatrice,CappBeatrice,CappVirgilio</v>
       </c>
     </row>
@@ -21936,7 +21951,7 @@
       <c r="M323" t="str">
         <v>AltoEnzo</v>
       </c>
-      <c r="Z323" t="str">
+      <c r="AA323" t="str">
         <v>AltoHolly</v>
       </c>
     </row>
@@ -21986,7 +22001,7 @@
       <c r="S324" t="str">
         <v>CappConsort</v>
       </c>
-      <c r="Z324" t="str">
+      <c r="AA324" t="str">
         <v>MontyDante</v>
       </c>
     </row>
@@ -22352,7 +22367,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z342"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AA342"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fix maritalStatus in data_FOR_CHECK.xlsx
</commit_message>
<xml_diff>
--- a/public/data_FOR_CHECK.xlsx
+++ b/public/data_FOR_CHECK.xlsx
@@ -14361,7 +14361,7 @@
         <v>Young Audlt</v>
       </c>
       <c r="H3" t="str">
-        <v>Married</v>
+        <v>{{Spouse</v>
       </c>
       <c r="I3" t="str">
         <v>Intelligence Researcher</v>
@@ -14574,7 +14574,7 @@
         <v>Elder</v>
       </c>
       <c r="H6" t="str">
-        <v>Divorced</v>
+        <v>{{Spouse</v>
       </c>
       <c r="I6" t="str">
         <v>Unemployed</v>
@@ -14914,7 +14914,7 @@
         <v>Young Audlt</v>
       </c>
       <c r="H11" t="str">
-        <v>Married</v>
+        <v>{{Spouse</v>
       </c>
       <c r="I11" t="str">
         <v>Caterer</v>

</xml_diff>

<commit_message>
fix maritalStatus parsing v2 in data_FOR_CHECK.xlsx
</commit_message>
<xml_diff>
--- a/public/data_FOR_CHECK.xlsx
+++ b/public/data_FOR_CHECK.xlsx
@@ -14361,7 +14361,7 @@
         <v>Young Audlt</v>
       </c>
       <c r="H3" t="str">
-        <v>{{Spouse</v>
+        <v>Married</v>
       </c>
       <c r="I3" t="str">
         <v>Intelligence Researcher</v>
@@ -14574,7 +14574,7 @@
         <v>Elder</v>
       </c>
       <c r="H6" t="str">
-        <v>{{Spouse</v>
+        <v>Divorced</v>
       </c>
       <c r="I6" t="str">
         <v>Unemployed</v>
@@ -14914,7 +14914,7 @@
         <v>Young Audlt</v>
       </c>
       <c r="H11" t="str">
-        <v>{{Spouse</v>
+        <v>Married</v>
       </c>
       <c r="I11" t="str">
         <v>Caterer</v>

</xml_diff>